<commit_message>
Honor closed collection-report decisions
Reuse existing Analysis tabs, suffix same-date extras with -2, pull
category amounts from column G into the weekly report, and keep a
single Thanksgiving name. Communion stays Midweek; email stays attach-only.

Co-authored-by: jayStar333 <jayStar333@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/wciclt-collection/samples/Collection Report 09.27.2026.xlsx
+++ b/wciclt-collection/samples/Collection Report 09.27.2026.xlsx
@@ -748,14 +748,14 @@
         </is>
       </c>
       <c r="B15" s="14" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="D15" s="13">
         <f>A15</f>
         <v/>
       </c>
       <c r="E15" s="14" t="n">
-        <v>0</v>
+        <v>385</v>
       </c>
     </row>
     <row r="16">
@@ -772,7 +772,7 @@
         <v/>
       </c>
       <c r="E16" s="14" t="n">
-        <v>0</v>
+        <v>1843.68</v>
       </c>
     </row>
     <row r="17">

</xml_diff>

<commit_message>
Fix weekly report service names that rendered invisible
openpyxl stored 6-digit RGB as transparent (00FFFFFF / 001F4E79), so
the sideways service labels vanished. Match the source reports: theme-1
black text on a light theme bar, and the 117-pt header row.

Co-authored-by: jayStar333 <jayStar333@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/wciclt-collection/samples/Collection Report 09.27.2026.xlsx
+++ b/wciclt-collection/samples/Collection Report 09.27.2026.xlsx
@@ -32,39 +32,45 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color theme="1"/>
       <sz val="24"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color theme="1"/>
       <sz val="18"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color theme="1"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
+      <color theme="1"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color theme="1"/>
       <sz val="14"/>
     </font>
     <font>
       <name val="Cambria"/>
+      <color theme="1"/>
       <sz val="14"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color theme="1"/>
       <sz val="26"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -78,12 +84,17 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="FFC6EFCE"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F4E79"/>
+        <fgColor theme="3" tint="0.5999938962981048"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.5999938962981048"/>
       </patternFill>
     </fill>
   </fills>
@@ -113,7 +124,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="18">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -122,6 +133,9 @@
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -527,16 +541,16 @@
     <col width="6.3" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
-    <row r="1" ht="12" customHeight="1"/>
-    <row r="2" ht="36" customHeight="1">
+    <row r="1" ht="15.75" customHeight="1"/>
+    <row r="2" ht="42.75" customHeight="1">
       <c r="A2" s="1" t="inlineStr">
         <is>
           <t>Winners Chapel International, Charlotte  Collection Report as at   09/23 - 09/27/2026</t>
         </is>
       </c>
     </row>
-    <row r="3" ht="8" customHeight="1"/>
-    <row r="4" ht="48" customHeight="1">
+    <row r="3" ht="6.75" customHeight="1"/>
+    <row r="4" ht="117" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Date:09.23.2026</t>
@@ -562,456 +576,456 @@
           <t>Sunday Service</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="F4" s="4" t="inlineStr">
         <is>
           <t>Sunday Service</t>
         </is>
       </c>
     </row>
     <row r="5" ht="36" customHeight="1">
-      <c r="A5" s="4" t="inlineStr">
+      <c r="A5" s="5" t="inlineStr">
         <is>
           <t>Recorded By:</t>
         </is>
       </c>
-      <c r="B5" s="4" t="inlineStr">
+      <c r="B5" s="5" t="inlineStr">
         <is>
           <t>Bro Ernest, Sis Sandra</t>
         </is>
       </c>
-      <c r="D5" s="4" t="inlineStr">
+      <c r="D5" s="5" t="inlineStr">
         <is>
           <t>Recorded By:</t>
         </is>
       </c>
-      <c r="E5" s="4" t="inlineStr">
+      <c r="E5" s="5" t="inlineStr">
         <is>
           <t>Bro Ernest, Sis Sandra</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="6" t="inlineStr">
         <is>
           <t>ATTENDANCE</t>
         </is>
       </c>
-      <c r="B6" s="6" t="n"/>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="B6" s="7" t="n"/>
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>ATTENDANCE</t>
         </is>
       </c>
-      <c r="E6" s="6" t="n"/>
+      <c r="E6" s="7" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="7" t="inlineStr">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>Men</t>
         </is>
       </c>
-      <c r="B7" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D7" s="7" t="inlineStr">
+      <c r="B7" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="8" t="inlineStr">
         <is>
           <t>Men</t>
         </is>
       </c>
-      <c r="E7" s="8" t="n">
+      <c r="E7" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>Women</t>
         </is>
       </c>
-      <c r="B8" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D8" s="7" t="inlineStr">
+      <c r="B8" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
         <is>
           <t>Women</t>
         </is>
       </c>
-      <c r="E8" s="8" t="n">
+      <c r="E8" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="7" t="inlineStr">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>Children</t>
         </is>
       </c>
-      <c r="B9" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D9" s="7" t="inlineStr">
+      <c r="B9" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="8" t="inlineStr">
         <is>
           <t>Children</t>
         </is>
       </c>
-      <c r="E9" s="8" t="n">
+      <c r="E9" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="7" t="inlineStr">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>First Timer</t>
         </is>
       </c>
-      <c r="B10" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D10" s="7" t="inlineStr">
+      <c r="B10" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
         <is>
           <t>First Timer</t>
         </is>
       </c>
-      <c r="E10" s="8" t="n">
+      <c r="E10" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="7" t="inlineStr">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>New Convert</t>
         </is>
       </c>
-      <c r="B11" s="8" t="n">
-        <v>0</v>
-      </c>
-      <c r="D11" s="7" t="inlineStr">
+      <c r="B11" s="9" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="8" t="inlineStr">
         <is>
           <t>New Convert</t>
         </is>
       </c>
-      <c r="E11" s="8" t="n">
+      <c r="E11" s="9" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B12" s="10">
+      <c r="B12" s="11">
         <f>SUM(B7:B9)</f>
         <v/>
       </c>
-      <c r="D12" s="9" t="inlineStr">
+      <c r="D12" s="10" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E12" s="10">
+      <c r="E12" s="11">
         <f>SUM(E7:E9)</f>
         <v/>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="11" t="inlineStr">
+      <c r="A13" s="12" t="inlineStr">
         <is>
           <t>COLLECTION</t>
         </is>
       </c>
-      <c r="B13" s="12" t="n"/>
-      <c r="D13" s="11" t="inlineStr">
+      <c r="B13" s="13" t="n"/>
+      <c r="D13" s="12" t="inlineStr">
         <is>
           <t>COLLECTION</t>
         </is>
       </c>
-      <c r="E13" s="12" t="n"/>
+      <c r="E13" s="13" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="6" t="inlineStr">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>Category</t>
         </is>
       </c>
-      <c r="B14" s="6" t="n"/>
-      <c r="D14" s="6">
+      <c r="B14" s="7" t="n"/>
+      <c r="D14" s="7">
         <f>A14</f>
         <v/>
       </c>
-      <c r="E14" s="6" t="n"/>
+      <c r="E14" s="7" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="13" t="inlineStr">
+      <c r="A15" s="14" t="inlineStr">
         <is>
           <t>Offering</t>
         </is>
       </c>
-      <c r="B15" s="14" t="n">
+      <c r="B15" s="15" t="n">
         <v>42</v>
       </c>
-      <c r="D15" s="13">
+      <c r="D15" s="14">
         <f>A15</f>
         <v/>
       </c>
-      <c r="E15" s="14" t="n">
+      <c r="E15" s="15" t="n">
         <v>385</v>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="13" t="inlineStr">
+      <c r="A16" s="14" t="inlineStr">
         <is>
           <t>Tithe</t>
         </is>
       </c>
-      <c r="B16" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D16" s="13">
+      <c r="B16" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="14">
         <f>A16</f>
         <v/>
       </c>
-      <c r="E16" s="14" t="n">
+      <c r="E16" s="15" t="n">
         <v>1843.68</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="13" t="inlineStr">
+      <c r="A17" s="14" t="inlineStr">
         <is>
           <t>Kingdom care Seed</t>
         </is>
       </c>
-      <c r="B17" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D17" s="13">
+      <c r="B17" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="14">
         <f>A17</f>
         <v/>
       </c>
-      <c r="E17" s="14" t="n">
+      <c r="E17" s="15" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="13" t="inlineStr">
+      <c r="A18" s="14" t="inlineStr">
         <is>
           <t>Sacrifice Seed</t>
         </is>
       </c>
-      <c r="B18" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D18" s="13">
+      <c r="B18" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="14">
         <f>A18</f>
         <v/>
       </c>
-      <c r="E18" s="14" t="n">
+      <c r="E18" s="15" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="13" t="inlineStr">
+      <c r="A19" s="14" t="inlineStr">
         <is>
           <t>SHILOH SACRIFICE</t>
         </is>
       </c>
-      <c r="B19" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D19" s="13">
+      <c r="B19" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="14">
         <f>A19</f>
         <v/>
       </c>
-      <c r="E19" s="14" t="n">
+      <c r="E19" s="15" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="13" t="inlineStr">
+      <c r="A20" s="14" t="inlineStr">
         <is>
           <t>End of Month Thanks-Giving</t>
         </is>
       </c>
-      <c r="B20" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D20" s="13">
+      <c r="B20" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="14">
         <f>A20</f>
         <v/>
       </c>
-      <c r="E20" s="14" t="n">
+      <c r="E20" s="15" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="13" t="inlineStr">
+      <c r="A21" s="14" t="inlineStr">
         <is>
           <t>Evangelism</t>
         </is>
       </c>
-      <c r="B21" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D21" s="13">
+      <c r="B21" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="14">
         <f>A21</f>
         <v/>
       </c>
-      <c r="E21" s="14" t="n">
+      <c r="E21" s="15" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="13" t="inlineStr">
+      <c r="A22" s="14" t="inlineStr">
         <is>
           <t>Building</t>
         </is>
       </c>
-      <c r="B22" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D22" s="13">
+      <c r="B22" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="14">
         <f>A22</f>
         <v/>
       </c>
-      <c r="E22" s="14" t="n">
+      <c r="E22" s="15" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="13" t="inlineStr">
+      <c r="A23" s="14" t="inlineStr">
         <is>
           <t>Welfare</t>
         </is>
       </c>
-      <c r="B23" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D23" s="13">
+      <c r="B23" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="14">
         <f>A23</f>
         <v/>
       </c>
-      <c r="E23" s="14" t="n">
+      <c r="E23" s="15" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="13" t="inlineStr">
+      <c r="A24" s="14" t="inlineStr">
         <is>
           <t>Chairs</t>
         </is>
       </c>
-      <c r="B24" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D24" s="13">
+      <c r="B24" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="14">
         <f>A24</f>
         <v/>
       </c>
-      <c r="E24" s="14" t="n">
+      <c r="E24" s="15" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="13" t="inlineStr">
+      <c r="A25" s="14" t="inlineStr">
         <is>
           <t>Bookstore</t>
         </is>
       </c>
-      <c r="B25" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D25" s="13">
+      <c r="B25" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="14">
         <f>A25</f>
         <v/>
       </c>
-      <c r="E25" s="14" t="n">
+      <c r="E25" s="15" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="13" t="inlineStr">
+      <c r="A26" s="14" t="inlineStr">
         <is>
           <t>Children's Dept</t>
         </is>
       </c>
-      <c r="B26" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D26" s="13">
+      <c r="B26" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="14">
         <f>A26</f>
         <v/>
       </c>
-      <c r="E26" s="14" t="n">
+      <c r="E26" s="15" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="13" t="inlineStr">
+      <c r="A27" s="14" t="inlineStr">
         <is>
           <t>Prophetic Offering</t>
         </is>
       </c>
-      <c r="B27" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D27" s="13">
+      <c r="B27" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="14">
         <f>A27</f>
         <v/>
       </c>
-      <c r="E27" s="14" t="n">
+      <c r="E27" s="15" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="13" t="inlineStr">
+      <c r="A28" s="14" t="inlineStr">
         <is>
           <t>Transportation</t>
         </is>
       </c>
-      <c r="B28" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D28" s="13">
+      <c r="B28" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="14">
         <f>A28</f>
         <v/>
       </c>
-      <c r="E28" s="14" t="n">
+      <c r="E28" s="15" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="13" t="inlineStr">
+      <c r="A29" s="14" t="inlineStr">
         <is>
           <t>Misc:</t>
         </is>
       </c>
-      <c r="B29" s="14" t="n">
-        <v>0</v>
-      </c>
-      <c r="D29" s="13">
+      <c r="B29" s="15" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="14">
         <f>A29</f>
         <v/>
       </c>
-      <c r="E29" s="14" t="n">
+      <c r="E29" s="15" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="15" t="inlineStr">
+      <c r="A30" s="16" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B30" s="16">
+      <c r="B30" s="17">
         <f>SUM(B15:B29)</f>
         <v/>
       </c>
-      <c r="D30" s="15" t="inlineStr">
+      <c r="D30" s="16" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="E30" s="16">
+      <c r="E30" s="17">
         <f>SUM(E15:E29)</f>
         <v/>
       </c>

</xml_diff>